<commit_message>
Add detailed content outlines to the topic video production sheet
New column G gives each of the 15 videos a recordable teaching
outline drawn from Sue's class script, the workbook, and the course
blueprint: hook, numbered teaching beats with her key lines quoted,
the pause-and-do cue where the blueprint places one, the workbook
mission, and a closing line. Week 5 rows remain marked draft pending
Alyson's content. YouTube links move to column H.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UMsCAA9Cstu5ucFmGvf6G2
</commit_message>
<xml_diff>
--- a/Thrive55_Topic_Video_Production_Sheet.xlsx
+++ b/Thrive55_Topic_Video_Production_Sheet.xlsx
@@ -2,23 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Topic Videos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Workbook Connections &amp; Tips" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,14 +28,72 @@
     <font>
       <name val="Georgia"/>
       <b val="1"/>
-      <color rgb="001B3A5B"/>
+      <color rgb="FF1B3A5B"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="0057635F"/>
+      <color rgb="FF57635F"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF187878"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B3A5B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FFA84A2E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF57635F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B3A5B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="FF1B3A5B"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="FF1B3A5B"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
@@ -44,54 +101,30 @@
       <sz val="11"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00187878"/>
-    </font>
-    <font>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001B3A5B"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00A84A2E"/>
       <sz val="10"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="0057635F"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001B3A5B"/>
-    </font>
-    <font>
-      <name val="Georgia"/>
-      <b val="1"/>
-      <color rgb="001B3A5B"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <name val="Georgia"/>
-      <b val="1"/>
-      <color rgb="001B3A5B"/>
-      <sz val="13"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF187878"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBF8F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBEDE7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -109,12 +142,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D2C7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D2C7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D2C7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D2C7"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -135,10 +183,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -187,7 +233,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -197,9 +242,25 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -562,615 +623,781 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="7.5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="7.44140625" customWidth="1" style="25" min="1" max="1"/>
+    <col width="26" customWidth="1" style="25" min="2" max="2"/>
+    <col width="34" customWidth="1" style="25" min="3" max="3"/>
+    <col width="10" customWidth="1" style="25" min="4" max="4"/>
+    <col width="46" customWidth="1" style="25" min="5" max="5"/>
+    <col width="60" customWidth="1" style="25" min="6" max="6"/>
+    <col width="100" customWidth="1" style="25" min="7" max="7"/>
+    <col width="30" customWidth="1" style="25" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Thrive 55+ Career Direction Program — Topic Video Production Sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>15 videos · record at your pace · paste each YouTube link in column G when uploaded (use Unlisted visibility) — I'll embed them in the app</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="1" ht="25.95" customHeight="1" s="25">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>Thrive 55+ Career Direction Program: Topic Video Production Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1" s="25">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>15 videos · record at your pace · paste each YouTube link in column G when uploaded (use Unlisted visibility): I'll embed them in the app</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1" s="25">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Topic Video Title</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Target Length (min)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Big Idea (one sentence)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Learning Objectives (learners will be able to…)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Detailed Content Outline (teach from this)</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>YouTube Link (paste here)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>Status / Notes</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="62" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="300" customHeight="1" s="25">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>V0.1</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Week 0 · Orientation</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>You're Not Done — Start Here</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>You're Not Done: Start Here</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Career direction is not one decision made in a panic; it is a method you can learn, repeat, and walk with a cohort beside you.</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>1. Describe the three parts of the Career Direction Method™ — name the strain, capture your value, investigate your options — and how the six weeks map to them.
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>1. Describe the three parts of the Career Direction Method: name the strain, capture your value, investigate your options: and how the six weeks map to them.
 2. Locate the workbook, the cohort space, and the weekly Learn → Do → Share loop.
 3. Write one intention for what you want to leave the program with.</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="G5" s="29" t="inlineStr">
+        <is>
+          <t>HOOK: "You are not done with nursing. You still have experience, judgment, value, and income needs. You just need a way of working that no longer leaves you dreading the next shift before the current one is over."
+1. Welcome to the cohort: you take this journey WITH other nurses, not alone. Introduce Sue and Alyson and the weekly rhythm: live webinar together, short lessons after, one workbook mission, then share with the cohort (Learn, Do, Share).
+2. Show the whole map: the method has three parts. Name the strain (Week 1). Capture your value (Week 2). Investigate your options (Weeks 3-4). Financial readiness with Alyson (Week 5). Your direction (Week 6).
+3. Point to the tools: the starting-point survey is the key that opens everything; the workbook saves their answers; Hope the coach is available anytime to talk it through.
+DO: Write one intention: "What do I want to leave this program with?"
+CLOSE: "We are not going to solve your whole career in six weeks. But you will leave with a way to start."</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="300" customHeight="1" s="25">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>V1.1</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Week 1 · Name the Strain</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Read the Work Before You Read the Job Board</t>
         </is>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>A career change does not start with a job title; it starts with understanding what the current work is asking of your body, attention, and capacity to adapt.</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>1. Explain why career direction begins with strain rather than with job titles.
 2. Distinguish “I still love nursing” from “this version of the work is sustainable for me.”</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="G6" s="30" t="inlineStr">
+        <is>
+          <t>HOOK: "Many nurses 55+ are not asking whether they still love nursing. They do. The harder question is whether their body and mind can keep carrying THIS version of the work until retirement."
+1. Career direction does NOT start with job titles. It does not begin with someone saying "Have you considered case management?" or "Maybe you could work in a clinic?" Those may be options, but they are not the starting point.
+2. The starting point is learning how to read the work. Three questions before any title: What is wearing you down? What do you bring with you? What direction is worth investigating next?
+3. Hold both truths: "I still love nursing" AND "this version of the work may not be sustainable for me." Neither cancels the other.
+4. Reframe: what you are feeling is information about the work, not a verdict about you.
+CLOSE: Next lesson we name the three specific forms that strain takes.</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="300" customHeight="1" s="25">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>V1.2</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Week 1 · Name the Strain</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>The Three Loads — Body, Interruption, Change</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>The Three Loads: Body, Interruption, Change</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Strain is not weakness or lost competence — it is information, and it arrives in three distinct forms you can name.</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Strain is not weakness or lost competence: it is information, and it arrives in three distinct forms you can name.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>1. Define body load, interruption load, and change load, and give one example of each from your own shifts.
 2. Sort your current stressors into the three loads.</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>TEACH the three loads, with the real examples for each:
+1. BODY LOAD: back pain, lifting, standing, bending, walking fast, reaching, transferring patients, working through pain, needing longer to recover between shifts. "Decades of nursing weigh heavily on a body. That does not mean you are weak. It means the current role may no longer be sustainable."
+2. INTERRUPTION LOAD: alarms, call lights, messages, questions, charting, new orders, unfinished tasks, open mental loops, constant task switching. The feeling of losing the thread because too many things pull at your attention at once. "That is workload information, not a competence issue." A nurse can be smart, capable, and experienced and still be worn down by constant interruption.
+3. CHANGE LOAD: new technology, new charting and EHR systems, policies, equipment, staffing models, changing expectations, limited onboarding. Continually adapting while still expected to perform at full speed.
+DO: Sort your own stressors into the three loads and name one example of each from your own shifts.
+CLOSE: "Next, we put numbers on them. Not to alarm you, to inform you."</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="300" customHeight="1" s="25">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>V1.3</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Week 1 · Name the Strain</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Score It, Don't Panic</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>Your highest strain score does not tell you to quit — it tells you where to look first.</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Your highest strain score does not tell you to quit: it tells you where to look first.</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>1. Rate each of the three loads on the 1–10 scale using the scoring guide.
 2. Interpret your highest score to name what the next role most needs to reduce.
 3. Reframe one strain from a fear into a piece of information.</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr"/>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>Pause-and-do lesson — say “pause me here” on camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="G8" s="31" t="inlineStr">
+        <is>
+          <t>TEACH the 1-10 scoring scale: 1-4 = not a current problem, or you notice it but can manage it. 5-6 = affecting your work or recovery. 7-8 = changing how you think about your future. 9-10 = may be threatening your ability to remain in your current role.
+KEY LINE: "The highest score does not tell you to panic. It tells you where to look first."
+WORKED CONTRASTS (teach all three):
+1. Body load 8, interruption load 3: career direction starts with less physically demanding roles.
+2. Interruption load 8: changing settings may not solve it if the next role still has constant task switching, heavy phone work, messages, and productivity pressure.
+3. Change load high: look closely at training required, onboarding quality, how technology-heavy the role is, and how fast independent performance is expected.
+PAUSE-AND-DO: "Pause me here." Score your three areas in the workbook (the lesson page opens the sliders right there).
+CLOSE: Reframe one strain out loud, from fear into information: "The point is not to label or limit yourself. It is to stop carrying the concern as fear and start looking at it as information."</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="n"/>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>Pause-and-do lesson: say “pause me here” on camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="300" customHeight="1" s="25">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>V2.1</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Week 2 · Capture Your Value</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Tell the Truth Without the Shame</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Naming what is getting harder is honest data, not a personal failing — and it must be kept separate from self-judgment.</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Naming what is getting harder is honest data, not a personal failing: and it must be kept separate from self-judgment.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>1. Name what is getting harder in your current role using non-punishing language.
 2. Differentiate an honest limitation from shame-based self-talk.</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="62" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>HOOK: Naming what is getting harder is honest data, not a personal failing.
+1. Name the categories where it gets harder: lifting, recovery after shifts, constant interruption, pace, technology, emotional wear.
+2. KEY LINE: "Tell yourself the truth. But do not turn the truth into shame."
+3. Teach the difference with paired examples: "I need longer to recover between shifts" is data. "I can't hack it anymore" is shame wearing a data costume. "New systems take me more time with good support" is data. "I'm too old for this" is shame.
+4. Data goes in the workbook; judgment does not. What you name honestly, you can solve. What you hide in shame keeps making the decision for you.
+DO: In the workbook, write what is getting harder using non-punishing language.
+CLOSE: "Next lesson is the other half of the truth: what you do WELL."</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="300" customHeight="1" s="25">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>V2.2</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Week 2 · Capture Your Value</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Your Ordinary Isn't Ordinary</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>The skills experienced nurses dismiss as “just the job” are hard-won, human, and exactly the ones automation cannot replace.</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>1. Identify at least five professional strengths built through years of nursing experience.
 2. Explain why judgment-and-relationship skills keep their value across different roles.
 3. Select one strength to carry into the next role.</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="16" t="inlineStr">
-        <is>
-          <t>Pause-and-do lesson — say “pause me here” on camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="G10" s="31" t="inlineStr">
+        <is>
+          <t>HOOK: "When you have done something for 20 or 30 years, the skills you use daily start to feel ordinary. That does not mean they ARE ordinary."
+1. Paint the evidence (use these images from the script): You have watched patients change before the monitor told the full story. You have heard the question underneath the question when a family member was scared. You have seen workflow break down before anyone called it a system problem. You read the room, the patient, the unit, the shift.
+2. Walk the skills list, slowly: reading patient and family cues; explaining complex information in plain language; organizing a messy situation; noticing safety concerns early; teaching a newer nurse without making them feel small; staying steady in difficult conditions; recognizing where workflow breaks down; communicating across roles; learning new systems with time and structure.
+3. CALLOUT: "These are not just compliments. They shape your nurse value. AI cannot duplicate these skills."
+PAUSE-AND-DO: "Pause me here." List five strengths you keep dismissing because they feel ordinary. Then pick ONE to carry into the next role.
+CLOSE: "Strain told you what to leave behind. Value tells you what comes with you."</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>Pause-and-do lesson: say “pause me here” on camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="300" customHeight="1" s="25">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>V3.1</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Reconnaissance Turns Fear Into Information</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Investigating options is not choosing a job today — it is gathering information so that fear stops making the decision for you.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Investigating options is not choosing a job today: it is gathering information so that fear stops making the decision for you.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>1. Explain the purpose of reconnaissance versus applying for jobs.
 2. Reframe two personal career fears as questions that can be investigated.</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12" ht="62" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="G11" s="29" t="inlineStr">
+        <is>
+          <t>HOOK: name the fears out loud (the learner should hear her own thoughts): What if I cannot learn the technology? What if I take less money? What if I leave the bedside and regret it? What if I apply and they do not want me? What if I am too old to start something different?
+1. Validate: "Those are real concerns. But fear alone does not give you good information. Reconnaissance does."
+2. Why the word reconnaissance: you are gathering intelligence, not committing. Investigating options is NOT choosing a final job today. It is deciding what direction is worth investigating next.
+3. Convert fear to a question you can answer (preview Concern-Question-Evidence): "I'll take too much of an income loss" becomes "What is the actual salary range and benefit package?" and the answer lives in postings, recruiters, and people doing the work.
+DO: Reframe two of your own career fears as questions you could investigate.
+CLOSE: Preview the three steps: study the work, ask people who know it, compare what you learn.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="300" customHeight="1" s="25">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>V3.2</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Study the Work — Read Postings Like a Detective</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="n">
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Study the Work: Read Postings Like a Detective</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>A job posting hides its real demands in one small paragraph; learning to read for it turns browsing into intelligence-gathering.</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>1. Set up job alerts and collect postings without applying.
 2. Extract the required skills, software, schedule, and physical demands from a posting.
 3. Locate the paragraph that describes what the person actually does all day.</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
-    </row>
-    <row r="13" ht="62" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="G12" s="30" t="inlineStr">
+        <is>
+          <t>STEP ONE of reconnaissance: study the work.
+1. Set up job alerts and let postings come to your email. "You do not have to apply. At first, you are studying. You are learning the language of the work."
+2. Read like a detective. Look for: repeated words and phrases; required vs preferred skills; specific software names; schedule expectations; physical requirements; whether the role is patient-facing, phone-heavy, chart-heavy, meeting-heavy, or technology-heavy.
+3. KEY MOVE: most postings are regulatory boilerplate. "Find the part, usually a small paragraph, that tells you what they actually need someone to do all day."
+4. TECH CONFIDENCE BEAT (important for this audience): track what you learn in a simple spreadsheet. If spreadsheets are new: download Google Sheets or Excel, ask ChatGPT "Help me set up a basic tracking spreadsheet," and follow the steps, or watch a short YouTube how-to. "Sometimes the hard part of technology is not understanding it. It is just getting started."
+DO: Set up one job alert and read five postings this week, no applying.
+CLOSE: "Postings tell you what employers say. Next lesson: what the work is actually like."</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="300" customHeight="1" s="25">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>V3.3</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Ask Three People This Week</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Three short conversations reveal what no posting can — and most people are glad to be asked.</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Three short conversations reveal what no posting can: and most people are glad to be asked.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>1. Identify three approachable people who know a role or setting of interest.
 2. Use the five reconnaissance questions to learn what a role is really like day to day.
 3. Ask “who else would be useful for me to talk to?” to open the next door.</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="G13" s="29" t="inlineStr">
+        <is>
+          <t>STEP TWO of reconnaissance: ask someone who knows the work.
+1. Right-size it: "Not fifty people. Not a giant networking project that feels awkward and overwhelming. Three people this week."
+2. Who counts: someone from another department, a former coworker, a nurse who changed roles, a recruiter, an educator, someone you meet in the cafeteria. "They do not have to be perfect contacts. They just need to know something useful."
+3. The questions: What does this job actually look like day to day? What part is harder than people realize? What technology do you use most? What skills mattered when you started? What is measured? What would you tell an experienced nurse considering this direction?
+4. THE DOOR-OPENER: always end with "Who else would be useful for me to talk to?" That one question opens the next door.
+5. Normalize the nerves: "The first time might feel uncomfortable. But most people appreciate being asked their thoughts. Usually people are kind and want to help."
+PAUSE-AND-DO: Log each conversation in the workbook: who, what you learned, who they suggested.
+CLOSE: "Three conversations will teach you what no posting can."</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+    </row>
+    <row r="14" ht="300" customHeight="1" s="25">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>V3.4</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Compare and Re-Score</t>
         </is>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>Better information changes the picture — a role you feared may open up, and a role that sounded easy may reveal red flags.</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Better information changes the picture: a role you feared may open up, and a role that sounded easy may reveal red flags.</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>1. Compare a researched role against your strain, value, income, and time needs.
 2. Re-score one strain area using new information and explain what changed.</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr"/>
-      <c r="H14" s="9" t="inlineStr"/>
-    </row>
-    <row r="15" ht="62" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>STEP THREE of reconnaissance: compare and re-score.
+1. "Your first score was based on what you knew then. Your second score is based on better information." Go back to your strain scores and weigh the role you researched against them.
+2. Three honest outcomes, all useful: a role you feared starts to look realistic; a role that sounded easy shows red flags; or you realize your biggest issue is not leaving nursing at all. "That is useful information."
+3. The compare questions: Does this role reduce the strain I am trying to solve? Does it use strengths I want to keep using? Does it introduce a different kind of strain I have not considered? Can it support the income I still need? How quickly could I realistically qualify, apply, and earn?
+4. The goal, said plainly: "You are finding a version of nursing that fits your body, brain, finances, and purpose better than the one you are in now."
+DO: Re-score one strain area using what a conversation or posting taught you, and note what changed.
+CLOSE: "Next: where to even look. Role categories, and the fine print."</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+    </row>
+    <row r="15" ht="300" customHeight="1" s="25">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>V3.5</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Role Categories, Red Flags, and Skill Gaps</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Categories are starting points, not answers; a red flag means look closer, and “I haven't done this lately” is not “I can't learn this.”</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>1. Name several nursing and nursing-adjacent role categories worth exploring.
 2. Evaluate a role's tradeoffs against your highest strain.
 3. Distinguish a genuine stop sign from a skill gap that can be rebuilt with time and practice.</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="G15" s="29" t="inlineStr">
+        <is>
+          <t>PART 1, CATEGORIES (starting points, not answers): outpatient / specialty clinic / medical office roles; case management / utilization review / CDI / quality; teaching, educating, mentoring; pre-admission and pre-authorization; remote triage and navigator roles; nursing-adjacent work such as writing, curriculum development, consulting, advocacy, community education. Full title list lives in the workbook and Roles Explorer.
+2. How to use a title: it is a search term, not a decision. Search several versions, read at least five postings. An unfamiliar title may describe work you already understand; a familiar title may hide demands you are trying to leave.
+PART 2, RED FLAGS AND TRADEOFFS: physically easier but cognitively heavier; less lifting but much more screen time; flexible schedule with tight productivity expectations; preserves nursing identity but does not solve your main strain; removes bedside work but removes the part of nursing you love; income takes too long to replace. KEY LINE: "A red flag does not always mean no. It means look closer before you leap."
+PART 3, SKILL GAP OR STOP SIGN: "Do not confuse 'I have not done this lately' with 'I cannot learn this.'" Skills can be rebuilt. Technology can be learned in pieces. New terminology becomes familiar. Interview language improves with practice. "Needing time, repetition, or support is different from being incapable."
+CLOSE: "You now have the whole reconnaissance toolkit. Next week: the money side, with Alyson."</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="300" customHeight="1" s="25">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>V5.1</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Week 5 · Financial Readiness</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Why Career and Money Belong Together</t>
         </is>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>A career decision is also a financial decision; readiness on both sides is what makes a change feel safe rather than reckless.</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>1. Explain why income, benefits, savings, and retirement timing belong in the same conversation as career direction.
 2. Identify the financial information to gather before making a change.</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr"/>
-      <c r="H16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17" ht="62" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="G16" s="30" t="inlineStr">
+        <is>
+          <t>BRIDGE from Sue (use her handoff line): "Career decisions do not happen separately from income, benefits, savings, and retirement timing. That is why career readiness and financial readiness belong in the same conversation."
+1. The feeling to address: a career change feels reckless when the money side is a fog; it feels safe when both sides are informed. Same fear-to-information move, applied to finances.
+2. Preview what Week 5 gathers (workbook handoff page): your current income; the minimum income your next role must support; your benefits inventory; and how quickly a new role must produce dependable income.
+3. No advice, no products: this is about knowing YOUR numbers and YOUR questions before any decision.
+DO: Open the Career-to-Financial Handoff page in the workbook and read it through once.
+NOTE: draft outline. Finalize wording and scope with Alyson's script before recording.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+    </row>
+    <row r="17" ht="300" customHeight="1" s="25">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>V5.2</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Week 5 · Financial Readiness</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>What to Gather — Income, Benefits, and Timing</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="n">
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>What to Gather: Income, Benefits, and Timing</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>You cannot weigh a new role honestly until you know your real number and how quickly a new role must produce income.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>1. Determine current income and the minimum income the next role must support.
 2. Inventory the core and additional benefits a change would affect.
 3. Estimate how quickly a new role needs to produce dependable income.</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="17" t="inlineStr">
-        <is>
-          <t>Draft — finalize with Alyson's content</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="G17" s="29" t="inlineStr">
+        <is>
+          <t>WHAT TO GATHER, three buckets (workbook handoff page):
+1. YOUR REAL NUMBER: current income, and an honest first estimate of the minimum income the next role must support. If you do not know it yet, that is a question to write down, not a reason to stop.
+2. BENEFITS INVENTORY, what a change would touch: core benefits (health insurance, retirement contribution or pension, paid time off, disability coverage) and additional benefits (life insurance, tuition support, FSA/HSA).
+3. TIMING: how quickly would a new role need to produce dependable income? Is there room for overlap, a bridge, or training time?
+4. Turn every unknown into a written question to bring into the financial discussion.
+DO: Complete the handoff page: income, benefits checklist, timing estimate, and your questions list.
+NOTE: draft outline. Finalize with Alyson's content and credentials for the lower third.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>Draft: finalize with Alyson's content</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="300" customHeight="1" s="25">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>V6.1</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Week 6 · Your Direction</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Choose One Informed Step</t>
         </is>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>You do not have to solve your whole career today; direction begins with a single, specific, informed step.</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>1. Select one concrete next step from the method (score, alert, five postings, one conversation, five strengths, start a tracker).
 2. Commit to when you will take it and what you expect to learn.</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr"/>
-      <c r="H18" s="16" t="inlineStr">
-        <is>
-          <t>Pause-and-do lesson — say “pause me here” on camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="G18" s="31" t="inlineStr">
+        <is>
+          <t>HOOK: "You do not have to solve your whole career today. You have to take the next informed step. That is where career direction begins."
+1. The menu (all steps count, pick ONE): score your three strain areas; set up one job alert; read five postings without applying; talk to one person; list five strengths you keep dismissing; start your job-research tracker; ask someone "Who else would be useful for me to talk to?"; bring your income questions into the financial discussion.
+2. Make it real: which step, by WHEN, and what do you expect to learn? A step without a date is a wish.
+3. Small is the strategy: one informed step this week beats a five-year plan you never start.
+PAUSE-AND-DO: "Pause me here." Choose your one step in the workbook, set the date, write what you expect to learn.
+CLOSE: "Bring your step to the cohort. Saying it out loud is half of keeping it."</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="n"/>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>Pause-and-do lesson: say “pause me here” on camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="300" customHeight="1" s="25">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>V6.2</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Week 6 · Your Direction</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Name the Strain. Capture Your Value. Investigate Your Options.</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>The method is repeatable — you now own a way to turn dread into information and information into your next step, for this decision and the next one.</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>The method is repeatable: you now own a way to turn dread into information and information into your next step, for this decision and the next one.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>1. Summarize your personal method: highest strain, value to carry forward, direction to investigate, and next step.
 2. Share your committed step with the cohort and name your ongoing support.</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr"/>
+      <c r="G19" s="29" t="inlineStr">
+        <is>
+          <t>THE CLOSE. Recap the whole method as a story:
+1. "You needed to stop carrying it as one large, unnamed fear." So you named the strain: body, interruption, change, scored 1 to 10, and your highest score told you where to look first.
+2. You captured your value: the skills that felt ordinary and are not, the ones AI cannot duplicate, and you chose what comes with you.
+3. You investigated your options: studied the work, asked three people, compared what you learned against your strain, your value, and your income needs.
+4. Personal method summary (have them say theirs): my highest strain, the problem my next role must solve, the value I carry forward, the direction I will investigate, the step I will take.
+5. KEY LINES, land them slowly: "You now have a way to start. A way to turn dread into information, and information into your next step." Then: "You are not less than. You are not done. You may just need a different way to do nursing."
+6. The method is repeatable: for this decision and the next one.
+DO: Complete the final survey to see your before-and-after, share your committed step with the cohort, and claim your certificate.
+CLOSE: Celebrate them. They finished something most nurses only think about.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n"/>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Total run time</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>~90 min</t>
         </is>
       </c>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
-      <c r="G20" s="18" t="n"/>
-      <c r="H20" s="18" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="n"/>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1183,332 +1410,334 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" style="25" min="1" max="1"/>
+    <col width="44" customWidth="1" style="25" min="2" max="2"/>
+    <col width="64" customWidth="1" style="25" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="25">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Where each video connects to the workbook</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C3" s="22" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>Connects to</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>V0.1</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>You're Not Done — Start Here</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>You're Not Done: Start Here</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>The Starting Point (workbook p.1–2)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>V1.1</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Read the Work Before You Read the Job Board</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>The Starting Point (workbook p.2)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>V1.2</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>The Three Loads — Body, Interruption, Change</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>The Three Loads: Body, Interruption, Change</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>Body / Interruption / Change load (workbook p.4–5)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>V1.3</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Score It, Don't Panic</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>Strain scores (workbook p.3–6) · PAUSE-AND-DO: score your three areas</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>V2.1</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Tell the Truth Without the Shame</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>What is getting harder (workbook p.6)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>V2.2</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Your Ordinary Isn't Ordinary</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>What do I still do well (workbook p.7) · PAUSE-AND-DO: five strengths</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>V3.1</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Reconnaissance Turns Fear Into Information</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>Options intro (workbook p.7–8)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>V3.2</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>Study the Work — Read Postings Like a Detective</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Study the Work: Read Postings Like a Detective</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>Study the Work (workbook p.8–9)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>V3.3</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Ask Three People This Week</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>Talk to Three People (workbook p.9)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>V3.4</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>Compare and Re-Score</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>Compare What You Learn (workbook p.10)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>V3.5</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>Role Categories, Red Flags, and Skill Gaps</t>
         </is>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>Roles, Red Flags &amp; Skill Gaps (workbook p.10–13)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>V5.1</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>Why Career and Money Belong Together</t>
         </is>
       </c>
-      <c r="C15" s="24" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>Career-to-Financial Handoff (workbook p.15)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+    <row r="16" ht="28.8" customHeight="1" s="25">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>V5.2</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>What to Gather — Income, Benefits, and Timing</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="inlineStr">
-        <is>
-          <t>Career-to-Financial Handoff (workbook p.15) · draft — finalize with Alyson's content</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>What to Gather: Income, Benefits, and Timing</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>Career-to-Financial Handoff (workbook p.15) · draft: finalize with Alyson's content</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28.8" customHeight="1" s="25">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>V6.1</t>
         </is>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>Choose One Informed Step</t>
         </is>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>Your Next Informed Step (workbook p.16) · PAUSE-AND-DO: one informed step</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+    <row r="18" ht="28.8" customHeight="1" s="25">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>V6.2</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>Name the Strain. Capture Your Value. Investigate Your Options.</t>
         </is>
       </c>
-      <c r="C18" s="24" t="inlineStr">
+      <c r="C18" s="21" t="inlineStr">
         <is>
           <t>My Career Direction Method (workbook p.16–17)</t>
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="A20" s="22" t="n"/>
+    </row>
+    <row r="21" ht="17.4" customHeight="1" s="25">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>Recording &amp; upload checklist</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>1. Upload each video to YouTube as UNLISTED (not private, not public) so it can embed in the app but won't appear in search.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>2. Keep on-screen text to phrases, not sentences — the workbook holds the detail (six or fewer short lines per slide).</t>
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>2. Keep on-screen text to phrases, not sentences: the workbook holds the detail (six or fewer short lines per slide).</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr">
-        <is>
-          <t>3. The three coral rows (V1.3, V2.2, V6.1) are pause-and-do lessons: say “pause me here if you want to do this now” — the app opens the matching workbook step right under the video.</t>
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>3. The three coral rows (V1.3, V2.2, V6.1) are pause-and-do lessons: say “pause me here if you want to do this now”: the app opens the matching workbook step right under the video.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>4. Paste the full YouTube link (e.g. https://youtu.be/XXXXXXXX) into column G of the Topic Videos sheet.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="25" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>5. Send the finished sheet back to me (or paste the links in chat) and I'll embed every video in its lesson page.</t>
         </is>

</xml_diff>

<commit_message>
Video outlines, gated Week 0 reading, coach kickoff lock, resources toolkit (#6)
Production sheet gains detailed teach-from-this outlines for all 15 videos. Beyond the Bedside becomes Week 0 gated program reading. Hope locks until the kickoff webinar (widget does not mount while locked). Resources page rebuilt as a reconnaissance toolkit: job research, interview preparation, and AI upskilling links curated for nurses 55+, with the method infographic gated behind the starting-point survey.
</commit_message>
<xml_diff>
--- a/Thrive55_Topic_Video_Production_Sheet.xlsx
+++ b/Thrive55_Topic_Video_Production_Sheet.xlsx
@@ -2,23 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Topic Videos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Workbook Connections &amp; Tips" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,14 +28,72 @@
     <font>
       <name val="Georgia"/>
       <b val="1"/>
-      <color rgb="001B3A5B"/>
+      <color rgb="FF1B3A5B"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="0057635F"/>
+      <color rgb="FF57635F"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF187878"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B3A5B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FFA84A2E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF57635F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1B3A5B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="FF1B3A5B"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="FF1B3A5B"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
@@ -44,54 +101,30 @@
       <sz val="11"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00187878"/>
-    </font>
-    <font>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001B3A5B"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00A84A2E"/>
       <sz val="10"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="0057635F"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001B3A5B"/>
-    </font>
-    <font>
-      <name val="Georgia"/>
-      <b val="1"/>
-      <color rgb="001B3A5B"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <name val="Georgia"/>
-      <b val="1"/>
-      <color rgb="001B3A5B"/>
-      <sz val="13"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF187878"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBF8F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBEDE7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -109,12 +142,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D2C7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D2C7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D2C7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D2C7"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -135,10 +183,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -187,7 +233,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -197,9 +242,25 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -562,615 +623,781 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="7.5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="7.44140625" customWidth="1" style="25" min="1" max="1"/>
+    <col width="26" customWidth="1" style="25" min="2" max="2"/>
+    <col width="34" customWidth="1" style="25" min="3" max="3"/>
+    <col width="10" customWidth="1" style="25" min="4" max="4"/>
+    <col width="46" customWidth="1" style="25" min="5" max="5"/>
+    <col width="60" customWidth="1" style="25" min="6" max="6"/>
+    <col width="100" customWidth="1" style="25" min="7" max="7"/>
+    <col width="30" customWidth="1" style="25" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Thrive 55+ Career Direction Program — Topic Video Production Sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>15 videos · record at your pace · paste each YouTube link in column G when uploaded (use Unlisted visibility) — I'll embed them in the app</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="1" ht="25.95" customHeight="1" s="25">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>Thrive 55+ Career Direction Program: Topic Video Production Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1" s="25">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>15 videos · record at your pace · paste each YouTube link in column G when uploaded (use Unlisted visibility): I'll embed them in the app</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1" s="25">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Topic Video Title</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Target Length (min)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Big Idea (one sentence)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Learning Objectives (learners will be able to…)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Detailed Content Outline (teach from this)</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>YouTube Link (paste here)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>Status / Notes</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="62" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="300" customHeight="1" s="25">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>V0.1</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Week 0 · Orientation</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>You're Not Done — Start Here</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>You're Not Done: Start Here</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Career direction is not one decision made in a panic; it is a method you can learn, repeat, and walk with a cohort beside you.</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>1. Describe the three parts of the Career Direction Method™ — name the strain, capture your value, investigate your options — and how the six weeks map to them.
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>1. Describe the three parts of the Career Direction Method: name the strain, capture your value, investigate your options: and how the six weeks map to them.
 2. Locate the workbook, the cohort space, and the weekly Learn → Do → Share loop.
 3. Write one intention for what you want to leave the program with.</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="G5" s="29" t="inlineStr">
+        <is>
+          <t>HOOK: "You are not done with nursing. You still have experience, judgment, value, and income needs. You just need a way of working that no longer leaves you dreading the next shift before the current one is over."
+1. Welcome to the cohort: you take this journey WITH other nurses, not alone. Introduce Sue and Alyson and the weekly rhythm: live webinar together, short lessons after, one workbook mission, then share with the cohort (Learn, Do, Share).
+2. Show the whole map: the method has three parts. Name the strain (Week 1). Capture your value (Week 2). Investigate your options (Weeks 3-4). Financial readiness with Alyson (Week 5). Your direction (Week 6).
+3. Point to the tools: the starting-point survey is the key that opens everything; the workbook saves their answers; Hope the coach is available anytime to talk it through.
+DO: Write one intention: "What do I want to leave this program with?"
+CLOSE: "We are not going to solve your whole career in six weeks. But you will leave with a way to start."</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="300" customHeight="1" s="25">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>V1.1</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Week 1 · Name the Strain</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Read the Work Before You Read the Job Board</t>
         </is>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>A career change does not start with a job title; it starts with understanding what the current work is asking of your body, attention, and capacity to adapt.</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>1. Explain why career direction begins with strain rather than with job titles.
 2. Distinguish “I still love nursing” from “this version of the work is sustainable for me.”</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="G6" s="30" t="inlineStr">
+        <is>
+          <t>HOOK: "Many nurses 55+ are not asking whether they still love nursing. They do. The harder question is whether their body and mind can keep carrying THIS version of the work until retirement."
+1. Career direction does NOT start with job titles. It does not begin with someone saying "Have you considered case management?" or "Maybe you could work in a clinic?" Those may be options, but they are not the starting point.
+2. The starting point is learning how to read the work. Three questions before any title: What is wearing you down? What do you bring with you? What direction is worth investigating next?
+3. Hold both truths: "I still love nursing" AND "this version of the work may not be sustainable for me." Neither cancels the other.
+4. Reframe: what you are feeling is information about the work, not a verdict about you.
+CLOSE: Next lesson we name the three specific forms that strain takes.</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="300" customHeight="1" s="25">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>V1.2</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Week 1 · Name the Strain</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>The Three Loads — Body, Interruption, Change</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>The Three Loads: Body, Interruption, Change</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Strain is not weakness or lost competence — it is information, and it arrives in three distinct forms you can name.</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Strain is not weakness or lost competence: it is information, and it arrives in three distinct forms you can name.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>1. Define body load, interruption load, and change load, and give one example of each from your own shifts.
 2. Sort your current stressors into the three loads.</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>TEACH the three loads, with the real examples for each:
+1. BODY LOAD: back pain, lifting, standing, bending, walking fast, reaching, transferring patients, working through pain, needing longer to recover between shifts. "Decades of nursing weigh heavily on a body. That does not mean you are weak. It means the current role may no longer be sustainable."
+2. INTERRUPTION LOAD: alarms, call lights, messages, questions, charting, new orders, unfinished tasks, open mental loops, constant task switching. The feeling of losing the thread because too many things pull at your attention at once. "That is workload information, not a competence issue." A nurse can be smart, capable, and experienced and still be worn down by constant interruption.
+3. CHANGE LOAD: new technology, new charting and EHR systems, policies, equipment, staffing models, changing expectations, limited onboarding. Continually adapting while still expected to perform at full speed.
+DO: Sort your own stressors into the three loads and name one example of each from your own shifts.
+CLOSE: "Next, we put numbers on them. Not to alarm you, to inform you."</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="300" customHeight="1" s="25">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>V1.3</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Week 1 · Name the Strain</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Score It, Don't Panic</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>Your highest strain score does not tell you to quit — it tells you where to look first.</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Your highest strain score does not tell you to quit: it tells you where to look first.</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>1. Rate each of the three loads on the 1–10 scale using the scoring guide.
 2. Interpret your highest score to name what the next role most needs to reduce.
 3. Reframe one strain from a fear into a piece of information.</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr"/>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>Pause-and-do lesson — say “pause me here” on camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="G8" s="31" t="inlineStr">
+        <is>
+          <t>TEACH the 1-10 scoring scale: 1-4 = not a current problem, or you notice it but can manage it. 5-6 = affecting your work or recovery. 7-8 = changing how you think about your future. 9-10 = may be threatening your ability to remain in your current role.
+KEY LINE: "The highest score does not tell you to panic. It tells you where to look first."
+WORKED CONTRASTS (teach all three):
+1. Body load 8, interruption load 3: career direction starts with less physically demanding roles.
+2. Interruption load 8: changing settings may not solve it if the next role still has constant task switching, heavy phone work, messages, and productivity pressure.
+3. Change load high: look closely at training required, onboarding quality, how technology-heavy the role is, and how fast independent performance is expected.
+PAUSE-AND-DO: "Pause me here." Score your three areas in the workbook (the lesson page opens the sliders right there).
+CLOSE: Reframe one strain out loud, from fear into information: "The point is not to label or limit yourself. It is to stop carrying the concern as fear and start looking at it as information."</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="n"/>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>Pause-and-do lesson: say “pause me here” on camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="300" customHeight="1" s="25">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>V2.1</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Week 2 · Capture Your Value</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Tell the Truth Without the Shame</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Naming what is getting harder is honest data, not a personal failing — and it must be kept separate from self-judgment.</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Naming what is getting harder is honest data, not a personal failing: and it must be kept separate from self-judgment.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>1. Name what is getting harder in your current role using non-punishing language.
 2. Differentiate an honest limitation from shame-based self-talk.</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="62" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>HOOK: Naming what is getting harder is honest data, not a personal failing.
+1. Name the categories where it gets harder: lifting, recovery after shifts, constant interruption, pace, technology, emotional wear.
+2. KEY LINE: "Tell yourself the truth. But do not turn the truth into shame."
+3. Teach the difference with paired examples: "I need longer to recover between shifts" is data. "I can't hack it anymore" is shame wearing a data costume. "New systems take me more time with good support" is data. "I'm too old for this" is shame.
+4. Data goes in the workbook; judgment does not. What you name honestly, you can solve. What you hide in shame keeps making the decision for you.
+DO: In the workbook, write what is getting harder using non-punishing language.
+CLOSE: "Next lesson is the other half of the truth: what you do WELL."</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="300" customHeight="1" s="25">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>V2.2</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Week 2 · Capture Your Value</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Your Ordinary Isn't Ordinary</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>The skills experienced nurses dismiss as “just the job” are hard-won, human, and exactly the ones automation cannot replace.</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>1. Identify at least five professional strengths built through years of nursing experience.
 2. Explain why judgment-and-relationship skills keep their value across different roles.
 3. Select one strength to carry into the next role.</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="16" t="inlineStr">
-        <is>
-          <t>Pause-and-do lesson — say “pause me here” on camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="G10" s="31" t="inlineStr">
+        <is>
+          <t>HOOK: "When you have done something for 20 or 30 years, the skills you use daily start to feel ordinary. That does not mean they ARE ordinary."
+1. Paint the evidence (use these images from the script): You have watched patients change before the monitor told the full story. You have heard the question underneath the question when a family member was scared. You have seen workflow break down before anyone called it a system problem. You read the room, the patient, the unit, the shift.
+2. Walk the skills list, slowly: reading patient and family cues; explaining complex information in plain language; organizing a messy situation; noticing safety concerns early; teaching a newer nurse without making them feel small; staying steady in difficult conditions; recognizing where workflow breaks down; communicating across roles; learning new systems with time and structure.
+3. CALLOUT: "These are not just compliments. They shape your nurse value. AI cannot duplicate these skills."
+PAUSE-AND-DO: "Pause me here." List five strengths you keep dismissing because they feel ordinary. Then pick ONE to carry into the next role.
+CLOSE: "Strain told you what to leave behind. Value tells you what comes with you."</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>Pause-and-do lesson: say “pause me here” on camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="300" customHeight="1" s="25">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>V3.1</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Reconnaissance Turns Fear Into Information</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Investigating options is not choosing a job today — it is gathering information so that fear stops making the decision for you.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Investigating options is not choosing a job today: it is gathering information so that fear stops making the decision for you.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>1. Explain the purpose of reconnaissance versus applying for jobs.
 2. Reframe two personal career fears as questions that can be investigated.</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12" ht="62" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="G11" s="29" t="inlineStr">
+        <is>
+          <t>HOOK: name the fears out loud (the learner should hear her own thoughts): What if I cannot learn the technology? What if I take less money? What if I leave the bedside and regret it? What if I apply and they do not want me? What if I am too old to start something different?
+1. Validate: "Those are real concerns. But fear alone does not give you good information. Reconnaissance does."
+2. Why the word reconnaissance: you are gathering intelligence, not committing. Investigating options is NOT choosing a final job today. It is deciding what direction is worth investigating next.
+3. Convert fear to a question you can answer (preview Concern-Question-Evidence): "I'll take too much of an income loss" becomes "What is the actual salary range and benefit package?" and the answer lives in postings, recruiters, and people doing the work.
+DO: Reframe two of your own career fears as questions you could investigate.
+CLOSE: Preview the three steps: study the work, ask people who know it, compare what you learn.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="300" customHeight="1" s="25">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>V3.2</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Study the Work — Read Postings Like a Detective</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="n">
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Study the Work: Read Postings Like a Detective</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>A job posting hides its real demands in one small paragraph; learning to read for it turns browsing into intelligence-gathering.</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>1. Set up job alerts and collect postings without applying.
 2. Extract the required skills, software, schedule, and physical demands from a posting.
 3. Locate the paragraph that describes what the person actually does all day.</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
-    </row>
-    <row r="13" ht="62" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="G12" s="30" t="inlineStr">
+        <is>
+          <t>STEP ONE of reconnaissance: study the work.
+1. Set up job alerts and let postings come to your email. "You do not have to apply. At first, you are studying. You are learning the language of the work."
+2. Read like a detective. Look for: repeated words and phrases; required vs preferred skills; specific software names; schedule expectations; physical requirements; whether the role is patient-facing, phone-heavy, chart-heavy, meeting-heavy, or technology-heavy.
+3. KEY MOVE: most postings are regulatory boilerplate. "Find the part, usually a small paragraph, that tells you what they actually need someone to do all day."
+4. TECH CONFIDENCE BEAT (important for this audience): track what you learn in a simple spreadsheet. If spreadsheets are new: download Google Sheets or Excel, ask ChatGPT "Help me set up a basic tracking spreadsheet," and follow the steps, or watch a short YouTube how-to. "Sometimes the hard part of technology is not understanding it. It is just getting started."
+DO: Set up one job alert and read five postings this week, no applying.
+CLOSE: "Postings tell you what employers say. Next lesson: what the work is actually like."</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="300" customHeight="1" s="25">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>V3.3</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Ask Three People This Week</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Three short conversations reveal what no posting can — and most people are glad to be asked.</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Three short conversations reveal what no posting can: and most people are glad to be asked.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>1. Identify three approachable people who know a role or setting of interest.
 2. Use the five reconnaissance questions to learn what a role is really like day to day.
 3. Ask “who else would be useful for me to talk to?” to open the next door.</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="G13" s="29" t="inlineStr">
+        <is>
+          <t>STEP TWO of reconnaissance: ask someone who knows the work.
+1. Right-size it: "Not fifty people. Not a giant networking project that feels awkward and overwhelming. Three people this week."
+2. Who counts: someone from another department, a former coworker, a nurse who changed roles, a recruiter, an educator, someone you meet in the cafeteria. "They do not have to be perfect contacts. They just need to know something useful."
+3. The questions: What does this job actually look like day to day? What part is harder than people realize? What technology do you use most? What skills mattered when you started? What is measured? What would you tell an experienced nurse considering this direction?
+4. THE DOOR-OPENER: always end with "Who else would be useful for me to talk to?" That one question opens the next door.
+5. Normalize the nerves: "The first time might feel uncomfortable. But most people appreciate being asked their thoughts. Usually people are kind and want to help."
+PAUSE-AND-DO: Log each conversation in the workbook: who, what you learned, who they suggested.
+CLOSE: "Three conversations will teach you what no posting can."</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+    </row>
+    <row r="14" ht="300" customHeight="1" s="25">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>V3.4</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Compare and Re-Score</t>
         </is>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>Better information changes the picture — a role you feared may open up, and a role that sounded easy may reveal red flags.</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Better information changes the picture: a role you feared may open up, and a role that sounded easy may reveal red flags.</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>1. Compare a researched role against your strain, value, income, and time needs.
 2. Re-score one strain area using new information and explain what changed.</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr"/>
-      <c r="H14" s="9" t="inlineStr"/>
-    </row>
-    <row r="15" ht="62" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>STEP THREE of reconnaissance: compare and re-score.
+1. "Your first score was based on what you knew then. Your second score is based on better information." Go back to your strain scores and weigh the role you researched against them.
+2. Three honest outcomes, all useful: a role you feared starts to look realistic; a role that sounded easy shows red flags; or you realize your biggest issue is not leaving nursing at all. "That is useful information."
+3. The compare questions: Does this role reduce the strain I am trying to solve? Does it use strengths I want to keep using? Does it introduce a different kind of strain I have not considered? Can it support the income I still need? How quickly could I realistically qualify, apply, and earn?
+4. The goal, said plainly: "You are finding a version of nursing that fits your body, brain, finances, and purpose better than the one you are in now."
+DO: Re-score one strain area using what a conversation or posting taught you, and note what changed.
+CLOSE: "Next: where to even look. Role categories, and the fine print."</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+    </row>
+    <row r="15" ht="300" customHeight="1" s="25">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>V3.5</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Weeks 3–4 · Investigate Your Options</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Role Categories, Red Flags, and Skill Gaps</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Categories are starting points, not answers; a red flag means look closer, and “I haven't done this lately” is not “I can't learn this.”</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>1. Name several nursing and nursing-adjacent role categories worth exploring.
 2. Evaluate a role's tradeoffs against your highest strain.
 3. Distinguish a genuine stop sign from a skill gap that can be rebuilt with time and practice.</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="G15" s="29" t="inlineStr">
+        <is>
+          <t>PART 1, CATEGORIES (starting points, not answers): outpatient / specialty clinic / medical office roles; case management / utilization review / CDI / quality; teaching, educating, mentoring; pre-admission and pre-authorization; remote triage and navigator roles; nursing-adjacent work such as writing, curriculum development, consulting, advocacy, community education. Full title list lives in the workbook and Roles Explorer.
+2. How to use a title: it is a search term, not a decision. Search several versions, read at least five postings. An unfamiliar title may describe work you already understand; a familiar title may hide demands you are trying to leave.
+PART 2, RED FLAGS AND TRADEOFFS: physically easier but cognitively heavier; less lifting but much more screen time; flexible schedule with tight productivity expectations; preserves nursing identity but does not solve your main strain; removes bedside work but removes the part of nursing you love; income takes too long to replace. KEY LINE: "A red flag does not always mean no. It means look closer before you leap."
+PART 3, SKILL GAP OR STOP SIGN: "Do not confuse 'I have not done this lately' with 'I cannot learn this.'" Skills can be rebuilt. Technology can be learned in pieces. New terminology becomes familiar. Interview language improves with practice. "Needing time, repetition, or support is different from being incapable."
+CLOSE: "You now have the whole reconnaissance toolkit. Next week: the money side, with Alyson."</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="300" customHeight="1" s="25">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>V5.1</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Week 5 · Financial Readiness</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Why Career and Money Belong Together</t>
         </is>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>A career decision is also a financial decision; readiness on both sides is what makes a change feel safe rather than reckless.</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>1. Explain why income, benefits, savings, and retirement timing belong in the same conversation as career direction.
 2. Identify the financial information to gather before making a change.</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr"/>
-      <c r="H16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17" ht="62" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="G16" s="30" t="inlineStr">
+        <is>
+          <t>BRIDGE from Sue (use her handoff line): "Career decisions do not happen separately from income, benefits, savings, and retirement timing. That is why career readiness and financial readiness belong in the same conversation."
+1. The feeling to address: a career change feels reckless when the money side is a fog; it feels safe when both sides are informed. Same fear-to-information move, applied to finances.
+2. Preview what Week 5 gathers (workbook handoff page): your current income; the minimum income your next role must support; your benefits inventory; and how quickly a new role must produce dependable income.
+3. No advice, no products: this is about knowing YOUR numbers and YOUR questions before any decision.
+DO: Open the Career-to-Financial Handoff page in the workbook and read it through once.
+NOTE: draft outline. Finalize wording and scope with Alyson's script before recording.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+    </row>
+    <row r="17" ht="300" customHeight="1" s="25">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>V5.2</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Week 5 · Financial Readiness</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>What to Gather — Income, Benefits, and Timing</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="n">
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>What to Gather: Income, Benefits, and Timing</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>You cannot weigh a new role honestly until you know your real number and how quickly a new role must produce income.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>1. Determine current income and the minimum income the next role must support.
 2. Inventory the core and additional benefits a change would affect.
 3. Estimate how quickly a new role needs to produce dependable income.</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="17" t="inlineStr">
-        <is>
-          <t>Draft — finalize with Alyson's content</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="G17" s="29" t="inlineStr">
+        <is>
+          <t>WHAT TO GATHER, three buckets (workbook handoff page):
+1. YOUR REAL NUMBER: current income, and an honest first estimate of the minimum income the next role must support. If you do not know it yet, that is a question to write down, not a reason to stop.
+2. BENEFITS INVENTORY, what a change would touch: core benefits (health insurance, retirement contribution or pension, paid time off, disability coverage) and additional benefits (life insurance, tuition support, FSA/HSA).
+3. TIMING: how quickly would a new role need to produce dependable income? Is there room for overlap, a bridge, or training time?
+4. Turn every unknown into a written question to bring into the financial discussion.
+DO: Complete the handoff page: income, benefits checklist, timing estimate, and your questions list.
+NOTE: draft outline. Finalize with Alyson's content and credentials for the lower third.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>Draft: finalize with Alyson's content</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="300" customHeight="1" s="25">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>V6.1</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Week 6 · Your Direction</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Choose One Informed Step</t>
         </is>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>You do not have to solve your whole career today; direction begins with a single, specific, informed step.</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>1. Select one concrete next step from the method (score, alert, five postings, one conversation, five strengths, start a tracker).
 2. Commit to when you will take it and what you expect to learn.</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr"/>
-      <c r="H18" s="16" t="inlineStr">
-        <is>
-          <t>Pause-and-do lesson — say “pause me here” on camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="G18" s="31" t="inlineStr">
+        <is>
+          <t>HOOK: "You do not have to solve your whole career today. You have to take the next informed step. That is where career direction begins."
+1. The menu (all steps count, pick ONE): score your three strain areas; set up one job alert; read five postings without applying; talk to one person; list five strengths you keep dismissing; start your job-research tracker; ask someone "Who else would be useful for me to talk to?"; bring your income questions into the financial discussion.
+2. Make it real: which step, by WHEN, and what do you expect to learn? A step without a date is a wish.
+3. Small is the strategy: one informed step this week beats a five-year plan you never start.
+PAUSE-AND-DO: "Pause me here." Choose your one step in the workbook, set the date, write what you expect to learn.
+CLOSE: "Bring your step to the cohort. Saying it out loud is half of keeping it."</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="n"/>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>Pause-and-do lesson: say “pause me here” on camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="300" customHeight="1" s="25">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>V6.2</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Week 6 · Your Direction</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Name the Strain. Capture Your Value. Investigate Your Options.</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>The method is repeatable — you now own a way to turn dread into information and information into your next step, for this decision and the next one.</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>The method is repeatable: you now own a way to turn dread into information and information into your next step, for this decision and the next one.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>1. Summarize your personal method: highest strain, value to carry forward, direction to investigate, and next step.
 2. Share your committed step with the cohort and name your ongoing support.</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr"/>
+      <c r="G19" s="29" t="inlineStr">
+        <is>
+          <t>THE CLOSE. Recap the whole method as a story:
+1. "You needed to stop carrying it as one large, unnamed fear." So you named the strain: body, interruption, change, scored 1 to 10, and your highest score told you where to look first.
+2. You captured your value: the skills that felt ordinary and are not, the ones AI cannot duplicate, and you chose what comes with you.
+3. You investigated your options: studied the work, asked three people, compared what you learned against your strain, your value, and your income needs.
+4. Personal method summary (have them say theirs): my highest strain, the problem my next role must solve, the value I carry forward, the direction I will investigate, the step I will take.
+5. KEY LINES, land them slowly: "You now have a way to start. A way to turn dread into information, and information into your next step." Then: "You are not less than. You are not done. You may just need a different way to do nursing."
+6. The method is repeatable: for this decision and the next one.
+DO: Complete the final survey to see your before-and-after, share your committed step with the cohort, and claim your certificate.
+CLOSE: Celebrate them. They finished something most nurses only think about.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n"/>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Total run time</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>~90 min</t>
         </is>
       </c>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
-      <c r="G20" s="18" t="n"/>
-      <c r="H20" s="18" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="n"/>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1183,332 +1410,334 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" style="25" min="1" max="1"/>
+    <col width="44" customWidth="1" style="25" min="2" max="2"/>
+    <col width="64" customWidth="1" style="25" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="25">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Where each video connects to the workbook</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C3" s="22" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>Connects to</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>V0.1</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>You're Not Done — Start Here</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>You're Not Done: Start Here</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>The Starting Point (workbook p.1–2)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>V1.1</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Read the Work Before You Read the Job Board</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>The Starting Point (workbook p.2)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>V1.2</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>The Three Loads — Body, Interruption, Change</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>The Three Loads: Body, Interruption, Change</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>Body / Interruption / Change load (workbook p.4–5)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>V1.3</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Score It, Don't Panic</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>Strain scores (workbook p.3–6) · PAUSE-AND-DO: score your three areas</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>V2.1</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Tell the Truth Without the Shame</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>What is getting harder (workbook p.6)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>V2.2</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Your Ordinary Isn't Ordinary</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>What do I still do well (workbook p.7) · PAUSE-AND-DO: five strengths</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>V3.1</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Reconnaissance Turns Fear Into Information</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>Options intro (workbook p.7–8)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>V3.2</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>Study the Work — Read Postings Like a Detective</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Study the Work: Read Postings Like a Detective</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>Study the Work (workbook p.8–9)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>V3.3</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Ask Three People This Week</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>Talk to Three People (workbook p.9)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>V3.4</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>Compare and Re-Score</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>Compare What You Learn (workbook p.10)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>V3.5</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>Role Categories, Red Flags, and Skill Gaps</t>
         </is>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>Roles, Red Flags &amp; Skill Gaps (workbook p.10–13)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>V5.1</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>Why Career and Money Belong Together</t>
         </is>
       </c>
-      <c r="C15" s="24" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>Career-to-Financial Handoff (workbook p.15)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+    <row r="16" ht="28.8" customHeight="1" s="25">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>V5.2</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>What to Gather — Income, Benefits, and Timing</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="inlineStr">
-        <is>
-          <t>Career-to-Financial Handoff (workbook p.15) · draft — finalize with Alyson's content</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>What to Gather: Income, Benefits, and Timing</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>Career-to-Financial Handoff (workbook p.15) · draft: finalize with Alyson's content</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28.8" customHeight="1" s="25">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>V6.1</t>
         </is>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>Choose One Informed Step</t>
         </is>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>Your Next Informed Step (workbook p.16) · PAUSE-AND-DO: one informed step</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+    <row r="18" ht="28.8" customHeight="1" s="25">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>V6.2</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>Name the Strain. Capture Your Value. Investigate Your Options.</t>
         </is>
       </c>
-      <c r="C18" s="24" t="inlineStr">
+      <c r="C18" s="21" t="inlineStr">
         <is>
           <t>My Career Direction Method (workbook p.16–17)</t>
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="A20" s="22" t="n"/>
+    </row>
+    <row r="21" ht="17.4" customHeight="1" s="25">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>Recording &amp; upload checklist</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>1. Upload each video to YouTube as UNLISTED (not private, not public) so it can embed in the app but won't appear in search.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>2. Keep on-screen text to phrases, not sentences — the workbook holds the detail (six or fewer short lines per slide).</t>
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>2. Keep on-screen text to phrases, not sentences: the workbook holds the detail (six or fewer short lines per slide).</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr">
-        <is>
-          <t>3. The three coral rows (V1.3, V2.2, V6.1) are pause-and-do lessons: say “pause me here if you want to do this now” — the app opens the matching workbook step right under the video.</t>
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>3. The three coral rows (V1.3, V2.2, V6.1) are pause-and-do lessons: say “pause me here if you want to do this now”: the app opens the matching workbook step right under the video.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>4. Paste the full YouTube link (e.g. https://youtu.be/XXXXXXXX) into column G of the Topic Videos sheet.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="25" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>5. Send the finished sheet back to me (or paste the links in chat) and I'll embed every video in its lesson page.</t>
         </is>

</xml_diff>